<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-05 Le pompon d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-05.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le ballon du pompon</t>
+          <t>Le pompon d'Aniss</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour d'immeuble, rampe, pierre mouillée, ballon rouge</t>
+          <t>entrée, classe, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aniss, papa, maman</t>
+          <t>Aniss, papa, maman, maîtresse</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut dire que le ballon est rouge comme son pompon. Il parle trop tôt. L'écho de la cour couvre. Il lève la main, il attend, puis papa l'entend.</t>
+          <t>Un nuage de lait pousse jusqu'au manteau. Sur le pompon rouge, un éclat de pompon brille. Aniss veut parler du rouge, maintenant. Il coupe papa : les mots se perdent. Il tire trop vite : la fermeture se coince. À l'école, sa phrase se cogne à la classe. Il refuse de foncer, lève la main, attend, dit le rouge. Merci vécu. Sur la laine, l'éclat de pompon tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le pompon rouge tape la rampe. La laine pique un peu les doigts. La cour sent la pierre mouillée. Un seau laisse une flaque ronde. Une gouttière cliquette, tout bas. Le ballon rouge attend près du mur. Il est un peu lisse, un peu chaud. Tu as vu le ballon ? Il est rouge, papa. Comme mon pompon. Je veux le dire. Et le tapoter. On va le dire, alors. En ce moment, papa parle à maman. Ils sont près de la porte. Leurs voix tapent les murs. Il est rouge ! Comme le pompon ! Les mots tapent les murs aussi. Personne ne se tourne. Le ballon reste contre le mur. Papa. Papa parle encore à maman. Aniss ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air. Le pompon pend, tout sage. L'écho s'arrête un peu. Papa se tourne. Tu voulais dire quelque chose ? Le ballon est rouge. Comme mon pompon. Je t'entends, maintenant. Je t'entends aussi. Aniss tapote le ballon. Le ballon tremble, tout doux. Il revient contre le genou. Il danse. Merci, Aniss. Tu as attendu. Et je t'ai entendu. Le caoutchouc sent un peu chaud. Le pompon reste sur le manteau. Tu veux encore un tapot ? Oui.</t>
+          <t>Un nuage de lait pousse jusqu'au manteau. Le pompon rouge tape la fermeture. La laine est rêche sous le pouce. L'air sent le lait chaud. Une tasse laisse un rond. Le rond brille sur le bois. Sur le pompon, un éclat de pompon brille. Il est petit, papa. C'est la laine, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le doudou attend sur la chaise. Le doudou a une oreille pliée. Je veux parler du rouge ! Pendant que je prends le sac ? Oui, tout de suite ! En ce moment, Aniss tire la fermeture. Le pompon rebondit contre le métal. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec le doudou. Papa, le rouge ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? Le pompon va partir. Aniss tire trop vite. La fermeture se coince. Le pompon penche, puis retombe. Oh. L'éclat de pompon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le manteau va sur tes épaules ? Oui, papa. Aniss glisse un bras, puis l'autre. La laine rêche touche le cou. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, le pas sonne sous les pieds. L'école sent le savon et le bois. Aniss s'assoit sur le tapis. Le tapis est doux sous les genoux. Le pompon reste sur le manteau. Ça sent les crayons. Une chaise grince près du mur. Un cube rouge est près du genou. Aniss le pousse un peu. La maîtresse parle près d'un ballon. Bonjour les enfants. Bonjour, maîtresse. Le ballon est rouge, un peu lisse. Il sent le caoutchouc. Le ballon est rouge, comme le pompon ! Ses mots se cognent à la classe. Personne ne comprend le rouge. Aniss referme la bouche. Il serre le manteau près du genou. Le soir, la porte s'ouvre. Ça sent le lait chaud. Te voilà, Aniss. Ton manteau est un peu froid. Viens près de la tasse. Aniss pose le manteau sur la chaise. Il s'assoit. Le ventre est serré, très petit. Il regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le pompon rouge tape la rampe. La laine pique un peu les doigts. La cour sent la pierre mouillée. Un seau laisse une flaque ronde. Une gouttière cliquette, tout bas. Le ballon rouge attend près du mur. Il est un peu lisse, un peu chaud. Tu as vu le ballon ? Il est rouge, papa. Comme mon pompon. Je veux le dire. Et le tapoter. On va le dire, alors. En ce moment, papa parle à maman. Ils sont près de la porte. Leurs voix tapent les murs. Il est rouge ! Comme le pompon ! Les mots tapent les murs aussi. Personne ne se tourne. Le ballon reste contre le mur. Papa. Papa parle encore à maman. Aniss ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air. Le pompon pend, tout sage. L'écho s'arrête un peu. Papa se tourne. Tu voulais dire quelque chose ? Le ballon est rouge. Comme mon pompon. Je t'entends, maintenant. Je t'entends aussi. Aniss tapote le ballon. Le ballon tremble, tout doux. Il revient contre le genou. Il danse. Merci, Aniss. Tu as attendu. Et je t'ai entendu. Le caoutchouc sent un peu chaud. Le pompon reste sur le manteau. Tu veux encore un tapot ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un nuage de lait pousse jusqu'au manteau. Le pompon rouge tape la fermeture. La laine est rêche sous le pouce. L'air sent le lait chaud. Une tasse laisse un rond. Le rond brille sur le bois. Sur le pompon, un &lt;emphasis level="moderate"&gt;éclat de pompon&lt;/emphasis&gt; brille. Il est petit, papa. C'est la laine, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le doudou attend sur la chaise. Le doudou a une oreille pliée. Je veux parler du rouge ! Pendant que je prends le sac ? Oui, tout de suite ! En ce moment, Aniss tire la fermeture. Le pompon rebondit contre le métal. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec le doudou. Papa, le rouge ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? Le pompon va partir. Aniss tire trop vite. La fermeture se coince. Le pompon penche, puis retombe. Oh. L'éclat de pompon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le manteau va sur tes épaules ? Oui, papa. Aniss glisse un bras, puis l'autre. La laine rêche touche le cou. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, le pas sonne sous les pieds. L'école sent le savon et le bois. Aniss s'assoit sur le tapis. Le tapis est doux sous les genoux. Le pompon reste sur le manteau. Ça sent les crayons. Une chaise grince près du mur. Un cube rouge est près du genou. Aniss le pousse un peu. La maîtresse parle près d'un ballon. Bonjour les enfants. Bonjour, maîtresse. Le ballon est rouge, un peu lisse. Il sent le caoutchouc. Le ballon est rouge, comme le pompon ! Ses mots se cognent à la classe. Personne ne comprend le rouge. Aniss referme la bouche. Il serre le manteau près du genou. Le soir, la porte s'ouvre. Ça sent le lait chaud. Te voilà, Aniss. Ton manteau est un peu froid. Viens près de la tasse. Aniss pose le manteau sur la chaise. Il s'assoit. Le ventre est serré, très petit. Il regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora arrive en classe avec papa. Papa dit au revoir. Flora s'assoit sur le tapis. La maîtresse pose une question. Flora a une idée. Elle lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Flora attend encore. Puis la maîtresse dit : Flora, c'est toi. Flora parle. Elle dit : le chat est gris. La maîtresse sourit. Le soir, papa demande. Flora dit : j'ai levé la main. J'ai su attendre. Puis parler, c'est après. Papa dit : tu as attendu. Puis tu as parlé.&lt;/slow&gt; [pause]</t>
+          <t>Un nuage de lait pousse jusqu'au manteau. Le pompon rouge tape la fermeture. La laine est rêche sous le pouce. L'air sent le lait chaud. Une tasse laisse un rond. Le rond brille sur le bois. Sur le pompon, un &lt;emphasis&gt;éclat de pompon&lt;/emphasis&gt; brille. Il est petit, papa. C'est la laine, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le doudou attend sur la chaise. Le doudou a une oreille pliée. Je veux parler du rouge ! Pendant que je prends le sac ? Oui, tout de suite ! En ce moment, Aniss tire la fermeture. Le pompon rebondit contre le métal. Papa parle à maman, près de la porte. Le cartable est près du banc. Oui, avec le doudou. Papa, le rouge ! Les mots d'Aniss se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose, Aniss ? Le pompon va partir. Aniss tire trop vite. La fermeture se coince. Le pompon penche, puis retombe. Oh. L'éclat de pompon tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le manteau va sur tes épaules ? Oui, papa. Aniss glisse un bras, puis l'autre. La laine rêche touche le cou. On y va ? On y va. Au revoir, maman. Au revoir, Aniss. Dehors, le pas sonne sous les pieds. L'école sent le savon et le bois. Aniss s'assoit sur le tapis. Le tapis est doux sous les genoux. Le pompon reste sur le manteau. Ça sent les crayons. Une chaise grince près du mur. Un cube rouge est près du genou. Aniss le pousse un peu. La maîtresse parle près d'un ballon. Bonjour les enfants. Bonjour, maîtresse. Le ballon est rouge, un peu lisse. Il sent le caoutchouc. Le ballon est rouge, comme le pompon ! Ses mots se cognent à la classe. Personne ne comprend le rouge. Aniss referme la bouche. Il serre le manteau près du genou. Le soir, la porte s'ouvre. Ça sent le lait chaud. Te voilà, Aniss. Ton manteau est un peu froid. Viens près de la tasse. Aniss pose le manteau sur la chaise. Il s'assoit. Le ventre est serré, très petit. Il regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de pompon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,56 +1324,89 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_parler_du_rouge_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le pompon rouge tape la rampe.
-narrateur|La laine pique un peu les doigts.
-narrateur|La cour sent la pierre mouillée.
-narrateur|Un seau laisse une flaque ronde.
-narrateur|Une gouttière cliquette, tout bas.
-narrateur|Le ballon rouge attend près du mur.
-narrateur|Il est un peu lisse, un peu chaud.
-papa|Tu as vu le ballon ?
-enfant-m|Il est rouge, papa.
-enfant-m|Comme mon pompon.
-enfant-m|Je veux le dire.
-enfant-m|Et le tapoter.
-papa|On va le dire, alors.
-narrateur|En ce moment, papa parle à maman.
-narrateur|Ils sont près de la porte.
-narrateur|Leurs voix tapent les murs.
-enfant-m|Il est rouge !
-enfant-m|Comme le pompon !
-narrateur|Les mots tapent les murs aussi.
-narrateur|Personne ne se tourne.
-narrateur|Le ballon reste contre le mur.
-enfant-m|Papa.
-narrateur|Papa parle encore à maman.
-narrateur|Aniss ferme la bouche.
-narrateur|Il lève la main, tout droit.
-narrateur|Sa main reste en l'air.
-narrateur|Le pompon pend, tout sage.
-narrateur|L'écho s'arrête un peu.
-narrateur|Papa se tourne.
-papa|Tu voulais dire quelque chose ?
-enfant-m|Le ballon est rouge.
-enfant-m|Comme mon pompon.
-papa|Je t'entends, maintenant.
-maman|Je t'entends aussi.
-narrateur|Aniss tapote le ballon.
-narrateur|Le ballon tremble, tout doux.
-narrateur|Il revient contre le genou.
-enfant-m|Il danse.
-papa|Merci, Aniss.
-papa|Tu as attendu.
-papa|Et je t'ai entendu.
-narrateur|Le caoutchouc sent un peu chaud.
+          <t>narrateur|Un nuage de lait pousse jusqu'au manteau.
+narrateur|Le pompon rouge tape la fermeture.
+narrateur|La laine est rêche sous le pouce.
+narrateur|L'air sent le lait chaud.
+narrateur|Une tasse laisse un rond.
+narrateur|Le rond brille sur le bois.
+narrateur|Sur le pompon, un éclat de pompon brille.
+enfant-m|Il est petit, papa.
+papa|C'est la laine, sous la lumière.
+narrateur|Papa tient la main d'Aniss.
+papa|Ta main est bien dans la mienne.
+maman|Le doudou attend sur la chaise.
+narrateur|Le doudou a une oreille pliée.
+enfant-m|Je veux parler du rouge !
+maman|Pendant que je prends le sac ?
+enfant-m|Oui, tout de suite !
+narrateur|En ce moment, Aniss tire la fermeture.
+narrateur|Le pompon rebondit contre le métal.
+narrateur|Papa parle à maman, près de la porte.
+papa|Le cartable est près du banc.
+maman|Oui, avec le doudou.
+enfant-m|Papa, le rouge !
+narrateur|Les mots d'Aniss se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Aniss ?
+enfant-m|Le pompon va partir.
+narrateur|Aniss tire trop vite.
+narrateur|La fermeture se coince.
+narrateur|Le pompon penche, puis retombe.
+enfant-m|Oh.
+narrateur|L'éclat de pompon tremble, puis tient.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Ça ne veut pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Le manteau va sur tes épaules ?
+enfant-m|Oui, papa.
+narrateur|Aniss glisse un bras, puis l'autre.
+narrateur|La laine rêche touche le cou.
+papa|On y va ?
+enfant-m|On y va.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Aniss.
+narrateur|Dehors, le pas sonne sous les pieds.
+narrateur|L'école sent le savon et le bois.
+narrateur|Aniss s'assoit sur le tapis.
+narrateur|Le tapis est doux sous les genoux.
 narrateur|Le pompon reste sur le manteau.
-maman|Tu veux encore un tapot ?
-enfant-m|Oui.</t>
+narrateur|Ça sent les crayons.
+narrateur|Une chaise grince près du mur.
+narrateur|Un cube rouge est près du genou.
+narrateur|Aniss le pousse un peu.
+narrateur|La maîtresse parle près d'un ballon.
+maitresse|Bonjour les enfants.
+enfant-m|Bonjour, maîtresse.
+narrateur|Le ballon est rouge, un peu lisse.
+narrateur|Il sent le caoutchouc.
+enfant-m|Le ballon est rouge, comme le pompon !
+narrateur|Ses mots se cognent à la classe.
+narrateur|Personne ne comprend le rouge.
+narrateur|Aniss referme la bouche.
+narrateur|Il serre le manteau près du genou.
+narrateur|Le soir, la porte s'ouvre.
+narrateur|Ça sent le lait chaud.
+papa|Te voilà, Aniss.
+papa|Ton manteau est un peu froid.
+maman|Viens près de la tasse.
+narrateur|Aniss pose le manteau sur la chaise.
+narrateur|Il s'assoit.
+narrateur|Le ventre est serré, très petit.
+narrateur|Il regarde papa.
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1410,12 +1443,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora veut parler. Que fait-elle d'abord ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1425,7 +1458,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>attendre | il attend | lever la main | la main</t>
+          <t>attendre | il attend | lever la main | la main | il lève la main | son tour | il attend son tour</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1440,7 +1473,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Personne ne l'entend. Que fait Aniss d'abord ?</t>
+          <t>Il lève la main et il attend. Que fait Aniss ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,7 +1511,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,10 +1519,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1537,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1540,13 +1577,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1556,7 +1593,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_attend_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1626,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le ballon revient, tout lent. Aniss le tapote encore. Il fait un petit floup. La pierre de la cour est froide. Une goutte tombe du seau. Il est rouge. Comme le pompon ? Oui. Tu m'as entendu. Oui. Quand l'écho s'est tu. Quand ta main était là. Maman pose le doudou sur une marche. Le doudou a une oreille pliée. Il t'attend, ce soir. Oui, maman. Aniss frotte le pompon au ballon. Laine et caoutchouc se touchent. Ils sont pareils, un peu ? Tous les deux rouges.</t>
+          <t>Aniss ouvre la bouche trop vite. Papa, le pompon. Papa n'a pas fini sa phrase. Le lait est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Sa bouche se referme. Les mains se posent à plat. Une main se lève, un peu. Aniss écoute la cuisine, un instant. Le manteau sèche près de la chaise. Papa pose sa tasse. Le lait fume un peu. Maman n'a pas fini non plus. Aniss attend que le silence arrive. Sur le pompon, l'éclat de pompon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. Le ballon était rouge. Comme mon pompon. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le ballon revient, tout lent. Aniss le tapote encore. Il fait un petit floup. La pierre de la cour est froide. Une goutte tombe du seau. Il est rouge. Comme le pompon ? Oui. Tu m'as entendu. Oui. Quand l'écho s'est tu. Quand ta main était là. Maman pose le doudou sur une marche. Le doudou a une oreille pliée. Il t'attend, ce soir. Oui, maman. Aniss frotte le pompon au ballon. Laine et caoutchouc se touchent. Ils sont pareils, un peu ? Tous les deux rouges.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss ouvre la bouche trop vite. Papa, le pompon. Papa n'a pas fini sa phrase. Le lait est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Sa bouche se referme. Les mains se posent à plat. Une main se lève, un peu. Aniss écoute la cuisine, un instant. Le manteau sèche près de la chaise. Papa pose sa tasse. Le lait fume un peu. Maman n'a pas fini non plus. Aniss attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur le pompon, l'éclat de pompon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. Le ballon était rouge. Comme mon pompon. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora a levé la main. Elle a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; parler, c'était son tour.&lt;/slow&gt; [pause]</t>
+          <t>Aniss ouvre la bouche trop vite. Papa, le pompon. Papa n'a pas fini sa phrase. Le lait est chaud, Aniss. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Sa bouche se referme. Les mains se posent à plat. Une main se lève, un peu. Aniss écoute la cuisine, un instant. Le manteau sèche près de la chaise. Papa pose sa tasse. Le lait fume un peu. Maman n'a pas fini non plus. Aniss attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur le pompon, l'éclat de pompon brille. Il est là. Je peux te montrer quelque chose ? Oui, nous t'écoutons. Le ballon était rouge. Comme mon pompon. Merci, Aniss. Papa a entendu toute la phrase. Tu as fini ta tasse ? Presque, maman. Le ventre d'Aniss se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1683,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1691,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,30 +1717,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>silence</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1749,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1724,35 +1761,48 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_leve_la_main_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le ballon revient, tout lent.
-narrateur|Aniss le tapote encore.
-narrateur|Il fait un petit floup.
-narrateur|La pierre de la cour est froide.
-narrateur|Une goutte tombe du seau.
-enfant-m|Il est rouge.
-papa|Comme le pompon ?
-enfant-m|Oui.
-enfant-m|Tu m'as entendu.
-papa|Oui.
-papa|Quand l'écho s'est tu.
-papa|Quand ta main était là.
-narrateur|Maman pose le doudou sur une marche.
-narrateur|Le doudou a une oreille pliée.
-maman|Il t'attend, ce soir.
-enfant-m|Oui, maman.
-narrateur|Aniss frotte le pompon au ballon.
-narrateur|Laine et caoutchouc se touchent.
-papa|Ils sont pareils, un peu ?
-enfant-m|Tous les deux rouges.</t>
+          <t>narrateur|Aniss ouvre la bouche trop vite.
+enfant-m|Papa, le pompon.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le lait est chaud, Aniss.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Aniss refuse de foncer.
+narrateur|Sa bouche se referme.
+narrateur|Les mains se posent à plat.
+narrateur|Une main se lève, un peu.
+narrateur|Aniss écoute la cuisine, un instant.
+papa|Le manteau sèche près de la chaise.
+narrateur|Papa pose sa tasse.
+maman|Le lait fume un peu.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Aniss attend que le silence arrive.
+narrateur|Sur le pompon, l'éclat de pompon brille.
+enfant-m|Il est là.
+enfant-m|Je peux te montrer quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Le ballon était rouge.
+enfant-m|Comme mon pompon.
+papa|Merci, Aniss.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as fini ta tasse ?
+enfant-m|Presque, maman.
+narrateur|Le ventre d'Aniss se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tasse,lait</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1829,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa reprend le manteau. Le pompon rebondit encore. On rentre ? Oui. Le ballon a dansé. Oui. Je t'ai entendu. Le doudou est dans le sac. Tu le prends ? Oui, maman. La flaque du seau reste ronde. La rampe est froide, maintenant. Le manteau sent la laine mouillée. Le doudou sent la maison.</t>
+          <t>Aniss prend le manteau sur la chaise. La laine est froide, un peu rêche. Je te montre le pompon. Tu lui fais une place ? Oui. Ici, sur le dossier. Aniss veut poser tout de suite. Il jette le manteau trop vite. Le manteau glisse du bois. Le pompon se cache sous le col. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la laine, un instant. Il écoute le clic de la fermeture. Il soulève le col, plus léger. Le pompon reparaît, bien rond. Il est là. On voit le rouge. Et le doudou, à côté ? Il a l'oreille pliée. Le doudou rejoint le manteau. Fffff. Aniss souffle sur le pompon.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa reprend le manteau. Le pompon rebondit encore. On rentre ? Oui. Le ballon a dansé. Oui. Je t'ai entendu. Le doudou est dans le sac. Tu le prends ? Oui, maman. La flaque du seau reste ronde. La rampe est froide, maintenant. Le manteau sent la laine mouillée. Le doudou sent la maison.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss prend le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; sur la chaise. La laine est froide, un peu rêche. Je te montre le pompon. Tu lui fais une place ? Oui. Ici, sur le dossier. Aniss veut poser tout de suite. Il jette le manteau trop vite. Le manteau glisse du bois. Le pompon se cache sous le col. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la laine, un instant. Il écoute le clic de la fermeture. Il soulève le col, plus léger. Le pompon reparaît, bien rond. Il est là. On voit le rouge. Et le doudou, à côté ? Il a l'oreille pliée. Le doudou rejoint le manteau. Fffff. Aniss souffle sur le pompon.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Flora range son cartable. Papa l'attend à la porte.&lt;/slow&gt; [pause]</t>
+          <t>Aniss prend le &lt;emphasis&gt;manteau&lt;/emphasis&gt; sur la chaise. La laine est froide, un peu rêche. Je te montre le pompon. Tu lui fais une place ? Oui. Ici, sur le dossier. Aniss veut poser tout de suite. Il jette le manteau trop vite. Le manteau glisse du bois. Le pompon se cache sous le col. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la laine, un instant. Il écoute le clic de la fermeture. Il soulève le col, plus léger. Le pompon reparaît, bien rond. Il est là. On voit le rouge. Et le doudou, à côté ? Il a l'oreille pliée. Le doudou rejoint le manteau. Fffff. Aniss souffle sur le pompon. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1836,7 +1886,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1844,10 +1894,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1868,28 +1918,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>manteau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1952,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1910,30 +1964,46 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_le_manteau; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa reprend le manteau.
-narrateur|Le pompon rebondit encore.
-papa|On rentre ?
+          <t>narrateur|Aniss prend le manteau sur la chaise.
+narrateur|La laine est froide, un peu rêche.
+enfant-m|Je te montre le pompon.
+papa|Tu lui fais une place ?
 enfant-m|Oui.
-enfant-m|Le ballon a dansé.
-papa|Oui.
-papa|Je t'ai entendu.
-maman|Le doudou est dans le sac.
-maman|Tu le prends ?
-enfant-m|Oui, maman.
-narrateur|La flaque du seau reste ronde.
-narrateur|La rampe est froide, maintenant.
-narrateur|Le manteau sent la laine mouillée.
-narrateur|Le doudou sent la maison.</t>
+enfant-m|Ici, sur le dossier.
+narrateur|Aniss veut poser tout de suite.
+narrateur|Il jette le manteau trop vite.
+narrateur|Le manteau glisse du bois.
+narrateur|Le pompon se cache sous le col.
+enfant-m|Oh.
+narrateur|Aniss s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Aniss refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe la laine, un instant.
+narrateur|Il écoute le clic de la fermeture.
+narrateur|Il soulève le col, plus léger.
+narrateur|Le pompon reparaît, bien rond.
+enfant-m|Il est là.
+maman|On voit le rouge.
+papa|Et le doudou, à côté ?
+enfant-m|Il a l'oreille pliée.
+narrateur|Le doudou rejoint le manteau.
+enfant-m|Fffff.
+narrateur|Aniss souffle sur le pompon.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>cartable,porte</t>
+          <t>manteau,pompon</t>
         </is>
       </c>
     </row>
@@ -1960,17 +2030,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le pompon tape encore la rampe. Tu m'as entendu. Oui. Le ballon reste contre le mur. La cour sent la pierre, calme.</t>
+          <t>Le manteau repose sur la chaise. Le pompon reste sur la fermeture. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le rouge. On est bien, ici. Le lait fume un peu, près de la fenêtre. Aniss glisse le pompon sans se presser. La laine repose contre le métal. On le voit, maman. Tu le vois sur le rouge ? Oui, l'éclat. Le soir reste dans l'air. L'éclat de pompon tient sur la laine.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le pompon tape encore la rampe. Tu m'as entendu. Oui. Le ballon reste contre le mur. La cour sent la pierre, calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le manteau repose sur la chaise. Le pompon reste sur la fermeture. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le rouge. On est bien, ici. Le lait fume un peu, près de la fenêtre. Aniss glisse le pompon sans se presser. La laine repose contre le métal. On le voit, maman. Tu le vois sur le rouge ? Oui, l'éclat. Le soir reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de pompon&lt;/emphasis&gt; tient sur la laine.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le manteau repose sur la chaise. Le pompon reste sur la fermeture. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le rouge. On est bien, ici. Le lait fume un peu, près de la fenêtre. Aniss glisse le pompon sans se presser. La laine repose contre le métal. On le voit, maman. Tu le vois sur le rouge ? Oui, l'éclat. Le soir reste dans l'air. L'&lt;emphasis&gt;éclat de pompon&lt;/emphasis&gt; tient sur la laine.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,18 +2087,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2037,12 +2107,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2121,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pompon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2144,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,28 +2157,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_laine; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le pompon tape encore la rampe.
-enfant-m|Tu m'as entendu.
-papa|Oui.
-narrateur|Le ballon reste contre le mur.
-narrateur|La cour sent la pierre, calme.</t>
+          <t>narrateur|Le manteau repose sur la chaise.
+narrateur|Le pompon reste sur la fermeture.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le rouge.
+maman|On est bien, ici.
+narrateur|Le lait fume un peu, près de la fenêtre.
+narrateur|Aniss glisse le pompon sans se presser.
+narrateur|La laine repose contre le métal.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le rouge ?
+enfant-m|Oui, l'éclat.
+narrateur|Le soir reste dans l'air.
+narrateur|L'éclat de pompon tient sur la laine.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>lait,pompon</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2189,6 +2281,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>